<commit_message>
Holiday tracker: month columns use the calculated (berry) header colour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C31xGpXxLcjXH3oTDRifkH
</commit_message>
<xml_diff>
--- a/products/holiday-hidden-cost-tracker/Holiday-Hidden-Cost-Tracker.xlsx
+++ b/products/holiday-hidden-cost-tracker/Holiday-Hidden-Cost-Tracker.xlsx
@@ -5678,23 +5678,23 @@
           <t>FLAG</t>
         </is>
       </c>
-      <c r="R5" s="27">
+      <c r="R5" s="19">
         <f>UPPER(TEXT(EDATE(Settings!$C$7,0),"mmm yyyy"))</f>
         <v/>
       </c>
-      <c r="S5" s="27">
+      <c r="S5" s="19">
         <f>UPPER(TEXT(EDATE(Settings!$C$7,1),"mmm yyyy"))</f>
         <v/>
       </c>
-      <c r="T5" s="27">
+      <c r="T5" s="19">
         <f>UPPER(TEXT(EDATE(Settings!$C$7,2),"mmm yyyy"))</f>
         <v/>
       </c>
-      <c r="U5" s="27">
+      <c r="U5" s="19">
         <f>UPPER(TEXT(EDATE(Settings!$C$7,3),"mmm yyyy"))</f>
         <v/>
       </c>
-      <c r="V5" s="27">
+      <c r="V5" s="19">
         <f>UPPER(TEXT(EDATE(Settings!$C$7,4),"mmm yyyy"))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Holiday tracker v1.1: Deal Check tab (xlsx, recalculated 0 errors); 3 Black Friday deal pins (v4)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C31xGpXxLcjXH3oTDRifkH
</commit_message>
<xml_diff>
--- a/products/holiday-hidden-cost-tracker/Holiday-Hidden-Cost-Tracker.xlsx
+++ b/products/holiday-hidden-cost-tracker/Holiday-Hidden-Cost-Tracker.xlsx
@@ -13,12 +13,14 @@
     <sheet name="Gift List" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Holiday Payments" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Free Trials" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Chart Data" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Deal Check" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Chart Data" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Gift List'!$B$5:$K$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Holiday Payments'!$B$5:$Q$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Free Trials'!$B$5:$L$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Deal Check'!$B$5:$P$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -123,6 +125,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <strike val="0"/>
+      <color rgb="00A7B2A3"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <strike val="0"/>
       <color rgb="00E0B05A"/>
       <sz val="22"/>
     </font>
@@ -188,13 +197,6 @@
       <strike val="0"/>
       <color rgb="005CC8B8"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <strike val="0"/>
-      <color rgb="00A7B2A3"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -501,48 +503,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf applyFill="1" numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf applyFill="1" applyFont="1" numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="171" fontId="13" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="171" fontId="14" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" indent="1"/>
     </xf>
-    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="14" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="16" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="14" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="17" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="9" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" indent="1"/>
     </xf>
-    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="17" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="18" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="169" fontId="17" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="169" fontId="18" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="16" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="10" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -566,7 +568,7 @@
     <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="167" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -596,22 +598,22 @@
     <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="21" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="22" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf applyFill="1" applyFont="1" numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf applyFill="1" applyFont="1" numFmtId="0" fontId="24" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,6 +696,9 @@
     </xf>
     <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1281,6 +1286,36 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>CheckMaybe</author>
+  </authors>
+  <commentList>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>The price you saw for the same item before the sale, for example the lowest price in the last 30 days. Leave it blank if you don't know; the verdict will ask for it.</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Your local sales tax rate. 0% if prices already include tax.</t>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0">
+      <text>
+        <t>Only if you'll pay on a plan. Leave blank if you pay in full.</t>
+      </text>
+    </comment>
+    <comment ref="P5" authorId="0" shapeId="0">
+      <text>
+        <t>Real deal: at least the 'good deal' % below the usual price, you need it, and the plan adds nothing. Not a deal: the sale price is not below the usual price.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -2940,7 +2975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3049,9 +3084,9 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="45" t="inlineStr">
-        <is>
-          <t>5. Dashboard: budget left, what your holiday plans add to January and February, the costliest plan, and trials to cancel.</t>
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Deal Check: before you buy a sale item, enter the sale price and the usual price (before the sale), tax, shipping and</t>
         </is>
       </c>
       <c r="C13" s="1" t="n"/>
@@ -3060,21 +3095,25 @@
       <c r="A14" s="1" t="n"/>
       <c r="B14" s="46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Use the filter buttons on each table's header row (or the filter bars above it in Google Sheets).</t>
+          <t xml:space="preserve">     the plan if you'd pay on one. The verdict tells you if it's a real deal, a small one, or not a deal at all.</t>
         </is>
       </c>
       <c r="C14" s="1" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="46" t="inlineStr"/>
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>5. Dashboard: budget left, what your holiday plans add to January and February, the costliest plan, and trials to cancel.</t>
+        </is>
+      </c>
       <c r="C15" s="1" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n"/>
       <c r="B16" s="46" t="inlineStr">
         <is>
-          <t>The example rows are made up. Replace or delete them.</t>
+          <t xml:space="preserve">   • Use the filter buttons on each table's header row (or the filter bars above it in Google Sheets).</t>
         </is>
       </c>
       <c r="C16" s="1" t="n"/>
@@ -3088,19 +3127,23 @@
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="46" t="inlineStr">
         <is>
-          <t>Estimates only. Not financial advice. Real APR is an estimate from your payment schedule and does not include fees charged separately.</t>
+          <t>The example rows are made up. Replace or delete them.</t>
         </is>
       </c>
       <c r="C18" s="1" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
-      <c r="B19" s="1" t="n"/>
+      <c r="B19" s="46" t="inlineStr"/>
       <c r="C19" s="1" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
-      <c r="B20" s="1" t="n"/>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t>Estimates only. Not financial advice. Real APR is an estimate from your payment schedule and does not include fees charged separately.</t>
+        </is>
+      </c>
       <c r="C20" s="1" t="n"/>
     </row>
     <row r="21">
@@ -3132,6 +3175,16 @@
       <c r="A26" s="1" t="n"/>
       <c r="B26" s="1" t="n"/>
       <c r="C26" s="1" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n"/>
+      <c r="B28" s="1" t="n"/>
+      <c r="C28" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8184,6 +8237,1162 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00E0B05A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="44" t="inlineStr">
+        <is>
+          <t>Deal Check</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="43" t="inlineStr">
+        <is>
+          <t>GOLD headers: you fill in   ·   BERRY headers: calculated for you</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="58">
+        <f>COUNT('Deal Check'!$M$6:$M$25)&amp;" items checked   ·   "&amp;COUNTIF('Deal Check'!$P$6:$P$25,"Real deal")&amp;" real deals   ·   "&amp;COUNTIF('Deal Check'!$P$6:$P$25,"Not a deal")&amp;" not a deal   ·   plans add "&amp;TEXT(SUM('Deal Check'!$O$6:$O$25),"$#,##0")</f>
+        <v/>
+      </c>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
+      <c r="P3" s="1" t="n"/>
+      <c r="Q3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="73" t="inlineStr">
+        <is>
+          <t>Good deal = at least</t>
+        </is>
+      </c>
+      <c r="M4" s="53" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N4" s="51" t="inlineStr">
+        <is>
+          <t>below the usual price</t>
+        </is>
+      </c>
+      <c r="O4" s="1" t="n"/>
+      <c r="P4" s="1" t="n"/>
+      <c r="Q4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>ITEM</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>STORE</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>SALE PRICE</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>USUAL PRICE</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>SALES TAX</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>SHIPPING</t>
+        </is>
+      </c>
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>PAY WITH</t>
+        </is>
+      </c>
+      <c r="I5" s="27" t="inlineStr">
+        <is>
+          <t>NUMBER OF PAYMENTS</t>
+        </is>
+      </c>
+      <c r="J5" s="27" t="inlineStr">
+        <is>
+          <t>EACH PAYMENT</t>
+        </is>
+      </c>
+      <c r="K5" s="27" t="inlineStr">
+        <is>
+          <t>NEED IT?</t>
+        </is>
+      </c>
+      <c r="L5" s="19" t="inlineStr">
+        <is>
+          <t>BELOW USUAL</t>
+        </is>
+      </c>
+      <c r="M5" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL AT CHECKOUT</t>
+        </is>
+      </c>
+      <c r="N5" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL ON THE PLAN</t>
+        </is>
+      </c>
+      <c r="O5" s="19" t="inlineStr">
+        <is>
+          <t>EXTRA ON THE PLAN</t>
+        </is>
+      </c>
+      <c r="P5" s="19" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+      <c r="Q5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="56" t="inlineStr">
+        <is>
+          <t>Noise-cancelling headphones</t>
+        </is>
+      </c>
+      <c r="C6" s="59" t="inlineStr">
+        <is>
+          <t>Store A</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="n">
+        <v>199</v>
+      </c>
+      <c r="E6" s="60" t="n">
+        <v>249</v>
+      </c>
+      <c r="F6" s="65" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G6" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="59" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="I6" s="63" t="n"/>
+      <c r="J6" s="60" t="n"/>
+      <c r="K6" s="59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L6" s="22">
+        <f>IF(AND(AND($B6&lt;&gt;"",ISNUMBER($D6)),N($E6)&gt;0),($E6-$D6)/$E6,"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="21">
+        <f>IF(AND($B6&lt;&gt;"",ISNUMBER($D6)),$D6*(1+N($F6))+N($G6),"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="21">
+        <f>IF(AND(AND($B6&lt;&gt;"",ISNUMBER($D6)),AND(N($I6)&gt;0,N($J6)&gt;0)),$I6*$J6,"")</f>
+        <v/>
+      </c>
+      <c r="O6" s="21">
+        <f>IF(ISNUMBER($N6),MAX(0,$N6-$M6),"")</f>
+        <v/>
+      </c>
+      <c r="P6" s="33">
+        <f>IF(NOT(AND($B6&lt;&gt;"",ISNUMBER($D6))),"",IF($K6="No","Skip it",IF(N($E6)=0,"Find the usual price",IF($D6&gt;=$E6,"Not a deal",IF(N($O6)&gt;0.005,"Deal, but the plan costs more",IF($L6&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="57" t="inlineStr">
+        <is>
+          <t>Air fryer</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>Store B</t>
+        </is>
+      </c>
+      <c r="D7" s="62" t="n">
+        <v>89</v>
+      </c>
+      <c r="E7" s="62" t="n">
+        <v>89</v>
+      </c>
+      <c r="F7" s="70" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G7" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="61" t="inlineStr">
+        <is>
+          <t>Cash / debit</t>
+        </is>
+      </c>
+      <c r="I7" s="68" t="n"/>
+      <c r="J7" s="62" t="n"/>
+      <c r="K7" s="61" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="L7" s="25">
+        <f>IF(AND(AND($B7&lt;&gt;"",ISNUMBER($D7)),N($E7)&gt;0),($E7-$D7)/$E7,"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="24">
+        <f>IF(AND($B7&lt;&gt;"",ISNUMBER($D7)),$D7*(1+N($F7))+N($G7),"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="24">
+        <f>IF(AND(AND($B7&lt;&gt;"",ISNUMBER($D7)),AND(N($I7)&gt;0,N($J7)&gt;0)),$I7*$J7,"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="24">
+        <f>IF(ISNUMBER($N7),MAX(0,$N7-$M7),"")</f>
+        <v/>
+      </c>
+      <c r="P7" s="35">
+        <f>IF(NOT(AND($B7&lt;&gt;"",ISNUMBER($D7))),"",IF($K7="No","Skip it",IF(N($E7)=0,"Find the usual price",IF($D7&gt;=$E7,"Not a deal",IF(N($O7)&gt;0.005,"Deal, but the plan costs more",IF($L7&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="1" t="n"/>
+      <c r="B8" s="56" t="inlineStr">
+        <is>
+          <t>55-inch TV</t>
+        </is>
+      </c>
+      <c r="C8" s="59" t="inlineStr">
+        <is>
+          <t>Store A</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="n">
+        <v>499</v>
+      </c>
+      <c r="E8" s="60" t="n">
+        <v>549</v>
+      </c>
+      <c r="F8" s="65" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G8" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="59" t="inlineStr">
+        <is>
+          <t>Store financing</t>
+        </is>
+      </c>
+      <c r="I8" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="60" t="n">
+        <v>49</v>
+      </c>
+      <c r="K8" s="59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L8" s="22">
+        <f>IF(AND(AND($B8&lt;&gt;"",ISNUMBER($D8)),N($E8)&gt;0),($E8-$D8)/$E8,"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="21">
+        <f>IF(AND($B8&lt;&gt;"",ISNUMBER($D8)),$D8*(1+N($F8))+N($G8),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="21">
+        <f>IF(AND(AND($B8&lt;&gt;"",ISNUMBER($D8)),AND(N($I8)&gt;0,N($J8)&gt;0)),$I8*$J8,"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="21">
+        <f>IF(ISNUMBER($N8),MAX(0,$N8-$M8),"")</f>
+        <v/>
+      </c>
+      <c r="P8" s="33">
+        <f>IF(NOT(AND($B8&lt;&gt;"",ISNUMBER($D8))),"",IF($K8="No","Skip it",IF(N($E8)=0,"Find the usual price",IF($D8&gt;=$E8,"Not a deal",IF(N($O8)&gt;0.005,"Deal, but the plan costs more",IF($L8&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="1" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="57" t="inlineStr">
+        <is>
+          <t>Smart watch</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>Store C</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="n">
+        <v>279</v>
+      </c>
+      <c r="E9" s="62" t="n">
+        <v>299</v>
+      </c>
+      <c r="F9" s="70" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G9" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="61" t="inlineStr">
+        <is>
+          <t>Pay-in-4</t>
+        </is>
+      </c>
+      <c r="I9" s="68" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="62" t="n">
+        <v>75.33</v>
+      </c>
+      <c r="K9" s="61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L9" s="25">
+        <f>IF(AND(AND($B9&lt;&gt;"",ISNUMBER($D9)),N($E9)&gt;0),($E9-$D9)/$E9,"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="24">
+        <f>IF(AND($B9&lt;&gt;"",ISNUMBER($D9)),$D9*(1+N($F9))+N($G9),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="24">
+        <f>IF(AND(AND($B9&lt;&gt;"",ISNUMBER($D9)),AND(N($I9)&gt;0,N($J9)&gt;0)),$I9*$J9,"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="24">
+        <f>IF(ISNUMBER($N9),MAX(0,$N9-$M9),"")</f>
+        <v/>
+      </c>
+      <c r="P9" s="35">
+        <f>IF(NOT(AND($B9&lt;&gt;"",ISNUMBER($D9))),"",IF($K9="No","Skip it",IF(N($E9)=0,"Find the usual price",IF($D9&gt;=$E9,"Not a deal",IF(N($O9)&gt;0.005,"Deal, but the plan costs more",IF($L9&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q9" s="1" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="56" t="inlineStr">
+        <is>
+          <t>Robot vacuum</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>Store B</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="n">
+        <v>159</v>
+      </c>
+      <c r="E10" s="60" t="n">
+        <v>299</v>
+      </c>
+      <c r="F10" s="65" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G10" s="60" t="n">
+        <v>15</v>
+      </c>
+      <c r="H10" s="59" t="inlineStr">
+        <is>
+          <t>Pay-in-4</t>
+        </is>
+      </c>
+      <c r="I10" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="60" t="n">
+        <v>46.68</v>
+      </c>
+      <c r="K10" s="59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L10" s="22">
+        <f>IF(AND(AND($B10&lt;&gt;"",ISNUMBER($D10)),N($E10)&gt;0),($E10-$D10)/$E10,"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="21">
+        <f>IF(AND($B10&lt;&gt;"",ISNUMBER($D10)),$D10*(1+N($F10))+N($G10),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="21">
+        <f>IF(AND(AND($B10&lt;&gt;"",ISNUMBER($D10)),AND(N($I10)&gt;0,N($J10)&gt;0)),$I10*$J10,"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="21">
+        <f>IF(ISNUMBER($N10),MAX(0,$N10-$M10),"")</f>
+        <v/>
+      </c>
+      <c r="P10" s="33">
+        <f>IF(NOT(AND($B10&lt;&gt;"",ISNUMBER($D10))),"",IF($K10="No","Skip it",IF(N($E10)=0,"Find the usual price",IF($D10&gt;=$E10,"Not a deal",IF(N($O10)&gt;0.005,"Deal, but the plan costs more",IF($L10&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="1" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="57" t="inlineStr">
+        <is>
+          <t>Electric scooter</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>Store C</t>
+        </is>
+      </c>
+      <c r="D11" s="62" t="n">
+        <v>349</v>
+      </c>
+      <c r="E11" s="62" t="n">
+        <v>449</v>
+      </c>
+      <c r="F11" s="70" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G11" s="62" t="n">
+        <v>25</v>
+      </c>
+      <c r="H11" s="61" t="inlineStr">
+        <is>
+          <t>Monthly BNPL</t>
+        </is>
+      </c>
+      <c r="I11" s="68" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="62" t="n">
+        <v>69</v>
+      </c>
+      <c r="K11" s="61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" s="25">
+        <f>IF(AND(AND($B11&lt;&gt;"",ISNUMBER($D11)),N($E11)&gt;0),($E11-$D11)/$E11,"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="24">
+        <f>IF(AND($B11&lt;&gt;"",ISNUMBER($D11)),$D11*(1+N($F11))+N($G11),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="24">
+        <f>IF(AND(AND($B11&lt;&gt;"",ISNUMBER($D11)),AND(N($I11)&gt;0,N($J11)&gt;0)),$I11*$J11,"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="24">
+        <f>IF(ISNUMBER($N11),MAX(0,$N11-$M11),"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="35">
+        <f>IF(NOT(AND($B11&lt;&gt;"",ISNUMBER($D11))),"",IF($K11="No","Skip it",IF(N($E11)=0,"Find the usual price",IF($D11&gt;=$E11,"Not a deal",IF(N($O11)&gt;0.005,"Deal, but the plan costs more",IF($L11&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="1" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="56" t="n"/>
+      <c r="C12" s="59" t="n"/>
+      <c r="D12" s="60" t="n"/>
+      <c r="E12" s="60" t="n"/>
+      <c r="F12" s="65" t="n"/>
+      <c r="G12" s="60" t="n"/>
+      <c r="H12" s="59" t="n"/>
+      <c r="I12" s="63" t="n"/>
+      <c r="J12" s="60" t="n"/>
+      <c r="K12" s="59" t="n"/>
+      <c r="L12" s="22">
+        <f>IF(AND(AND($B12&lt;&gt;"",ISNUMBER($D12)),N($E12)&gt;0),($E12-$D12)/$E12,"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="21">
+        <f>IF(AND($B12&lt;&gt;"",ISNUMBER($D12)),$D12*(1+N($F12))+N($G12),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="21">
+        <f>IF(AND(AND($B12&lt;&gt;"",ISNUMBER($D12)),AND(N($I12)&gt;0,N($J12)&gt;0)),$I12*$J12,"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="21">
+        <f>IF(ISNUMBER($N12),MAX(0,$N12-$M12),"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="33">
+        <f>IF(NOT(AND($B12&lt;&gt;"",ISNUMBER($D12))),"",IF($K12="No","Skip it",IF(N($E12)=0,"Find the usual price",IF($D12&gt;=$E12,"Not a deal",IF(N($O12)&gt;0.005,"Deal, but the plan costs more",IF($L12&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="1" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="1" t="n"/>
+      <c r="B13" s="57" t="n"/>
+      <c r="C13" s="61" t="n"/>
+      <c r="D13" s="62" t="n"/>
+      <c r="E13" s="62" t="n"/>
+      <c r="F13" s="70" t="n"/>
+      <c r="G13" s="62" t="n"/>
+      <c r="H13" s="61" t="n"/>
+      <c r="I13" s="68" t="n"/>
+      <c r="J13" s="62" t="n"/>
+      <c r="K13" s="61" t="n"/>
+      <c r="L13" s="25">
+        <f>IF(AND(AND($B13&lt;&gt;"",ISNUMBER($D13)),N($E13)&gt;0),($E13-$D13)/$E13,"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="24">
+        <f>IF(AND($B13&lt;&gt;"",ISNUMBER($D13)),$D13*(1+N($F13))+N($G13),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="24">
+        <f>IF(AND(AND($B13&lt;&gt;"",ISNUMBER($D13)),AND(N($I13)&gt;0,N($J13)&gt;0)),$I13*$J13,"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="24">
+        <f>IF(ISNUMBER($N13),MAX(0,$N13-$M13),"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="35">
+        <f>IF(NOT(AND($B13&lt;&gt;"",ISNUMBER($D13))),"",IF($K13="No","Skip it",IF(N($E13)=0,"Find the usual price",IF($D13&gt;=$E13,"Not a deal",IF(N($O13)&gt;0.005,"Deal, but the plan costs more",IF($L13&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="1" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="56" t="n"/>
+      <c r="C14" s="59" t="n"/>
+      <c r="D14" s="60" t="n"/>
+      <c r="E14" s="60" t="n"/>
+      <c r="F14" s="65" t="n"/>
+      <c r="G14" s="60" t="n"/>
+      <c r="H14" s="59" t="n"/>
+      <c r="I14" s="63" t="n"/>
+      <c r="J14" s="60" t="n"/>
+      <c r="K14" s="59" t="n"/>
+      <c r="L14" s="22">
+        <f>IF(AND(AND($B14&lt;&gt;"",ISNUMBER($D14)),N($E14)&gt;0),($E14-$D14)/$E14,"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="21">
+        <f>IF(AND($B14&lt;&gt;"",ISNUMBER($D14)),$D14*(1+N($F14))+N($G14),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="21">
+        <f>IF(AND(AND($B14&lt;&gt;"",ISNUMBER($D14)),AND(N($I14)&gt;0,N($J14)&gt;0)),$I14*$J14,"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="21">
+        <f>IF(ISNUMBER($N14),MAX(0,$N14-$M14),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="33">
+        <f>IF(NOT(AND($B14&lt;&gt;"",ISNUMBER($D14))),"",IF($K14="No","Skip it",IF(N($E14)=0,"Find the usual price",IF($D14&gt;=$E14,"Not a deal",IF(N($O14)&gt;0.005,"Deal, but the plan costs more",IF($L14&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="1" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="57" t="n"/>
+      <c r="C15" s="61" t="n"/>
+      <c r="D15" s="62" t="n"/>
+      <c r="E15" s="62" t="n"/>
+      <c r="F15" s="70" t="n"/>
+      <c r="G15" s="62" t="n"/>
+      <c r="H15" s="61" t="n"/>
+      <c r="I15" s="68" t="n"/>
+      <c r="J15" s="62" t="n"/>
+      <c r="K15" s="61" t="n"/>
+      <c r="L15" s="25">
+        <f>IF(AND(AND($B15&lt;&gt;"",ISNUMBER($D15)),N($E15)&gt;0),($E15-$D15)/$E15,"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="24">
+        <f>IF(AND($B15&lt;&gt;"",ISNUMBER($D15)),$D15*(1+N($F15))+N($G15),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="24">
+        <f>IF(AND(AND($B15&lt;&gt;"",ISNUMBER($D15)),AND(N($I15)&gt;0,N($J15)&gt;0)),$I15*$J15,"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="24">
+        <f>IF(ISNUMBER($N15),MAX(0,$N15-$M15),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="35">
+        <f>IF(NOT(AND($B15&lt;&gt;"",ISNUMBER($D15))),"",IF($K15="No","Skip it",IF(N($E15)=0,"Find the usual price",IF($D15&gt;=$E15,"Not a deal",IF(N($O15)&gt;0.005,"Deal, but the plan costs more",IF($L15&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q15" s="1" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="56" t="n"/>
+      <c r="C16" s="59" t="n"/>
+      <c r="D16" s="60" t="n"/>
+      <c r="E16" s="60" t="n"/>
+      <c r="F16" s="65" t="n"/>
+      <c r="G16" s="60" t="n"/>
+      <c r="H16" s="59" t="n"/>
+      <c r="I16" s="63" t="n"/>
+      <c r="J16" s="60" t="n"/>
+      <c r="K16" s="59" t="n"/>
+      <c r="L16" s="22">
+        <f>IF(AND(AND($B16&lt;&gt;"",ISNUMBER($D16)),N($E16)&gt;0),($E16-$D16)/$E16,"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="21">
+        <f>IF(AND($B16&lt;&gt;"",ISNUMBER($D16)),$D16*(1+N($F16))+N($G16),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="21">
+        <f>IF(AND(AND($B16&lt;&gt;"",ISNUMBER($D16)),AND(N($I16)&gt;0,N($J16)&gt;0)),$I16*$J16,"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="21">
+        <f>IF(ISNUMBER($N16),MAX(0,$N16-$M16),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="33">
+        <f>IF(NOT(AND($B16&lt;&gt;"",ISNUMBER($D16))),"",IF($K16="No","Skip it",IF(N($E16)=0,"Find the usual price",IF($D16&gt;=$E16,"Not a deal",IF(N($O16)&gt;0.005,"Deal, but the plan costs more",IF($L16&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="1" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="57" t="n"/>
+      <c r="C17" s="61" t="n"/>
+      <c r="D17" s="62" t="n"/>
+      <c r="E17" s="62" t="n"/>
+      <c r="F17" s="70" t="n"/>
+      <c r="G17" s="62" t="n"/>
+      <c r="H17" s="61" t="n"/>
+      <c r="I17" s="68" t="n"/>
+      <c r="J17" s="62" t="n"/>
+      <c r="K17" s="61" t="n"/>
+      <c r="L17" s="25">
+        <f>IF(AND(AND($B17&lt;&gt;"",ISNUMBER($D17)),N($E17)&gt;0),($E17-$D17)/$E17,"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="24">
+        <f>IF(AND($B17&lt;&gt;"",ISNUMBER($D17)),$D17*(1+N($F17))+N($G17),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="24">
+        <f>IF(AND(AND($B17&lt;&gt;"",ISNUMBER($D17)),AND(N($I17)&gt;0,N($J17)&gt;0)),$I17*$J17,"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="24">
+        <f>IF(ISNUMBER($N17),MAX(0,$N17-$M17),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="35">
+        <f>IF(NOT(AND($B17&lt;&gt;"",ISNUMBER($D17))),"",IF($K17="No","Skip it",IF(N($E17)=0,"Find the usual price",IF($D17&gt;=$E17,"Not a deal",IF(N($O17)&gt;0.005,"Deal, but the plan costs more",IF($L17&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q17" s="1" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="56" t="n"/>
+      <c r="C18" s="59" t="n"/>
+      <c r="D18" s="60" t="n"/>
+      <c r="E18" s="60" t="n"/>
+      <c r="F18" s="65" t="n"/>
+      <c r="G18" s="60" t="n"/>
+      <c r="H18" s="59" t="n"/>
+      <c r="I18" s="63" t="n"/>
+      <c r="J18" s="60" t="n"/>
+      <c r="K18" s="59" t="n"/>
+      <c r="L18" s="22">
+        <f>IF(AND(AND($B18&lt;&gt;"",ISNUMBER($D18)),N($E18)&gt;0),($E18-$D18)/$E18,"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="21">
+        <f>IF(AND($B18&lt;&gt;"",ISNUMBER($D18)),$D18*(1+N($F18))+N($G18),"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="21">
+        <f>IF(AND(AND($B18&lt;&gt;"",ISNUMBER($D18)),AND(N($I18)&gt;0,N($J18)&gt;0)),$I18*$J18,"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="21">
+        <f>IF(ISNUMBER($N18),MAX(0,$N18-$M18),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="33">
+        <f>IF(NOT(AND($B18&lt;&gt;"",ISNUMBER($D18))),"",IF($K18="No","Skip it",IF(N($E18)=0,"Find the usual price",IF($D18&gt;=$E18,"Not a deal",IF(N($O18)&gt;0.005,"Deal, but the plan costs more",IF($L18&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q18" s="1" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="57" t="n"/>
+      <c r="C19" s="61" t="n"/>
+      <c r="D19" s="62" t="n"/>
+      <c r="E19" s="62" t="n"/>
+      <c r="F19" s="70" t="n"/>
+      <c r="G19" s="62" t="n"/>
+      <c r="H19" s="61" t="n"/>
+      <c r="I19" s="68" t="n"/>
+      <c r="J19" s="62" t="n"/>
+      <c r="K19" s="61" t="n"/>
+      <c r="L19" s="25">
+        <f>IF(AND(AND($B19&lt;&gt;"",ISNUMBER($D19)),N($E19)&gt;0),($E19-$D19)/$E19,"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="24">
+        <f>IF(AND($B19&lt;&gt;"",ISNUMBER($D19)),$D19*(1+N($F19))+N($G19),"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="24">
+        <f>IF(AND(AND($B19&lt;&gt;"",ISNUMBER($D19)),AND(N($I19)&gt;0,N($J19)&gt;0)),$I19*$J19,"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="24">
+        <f>IF(ISNUMBER($N19),MAX(0,$N19-$M19),"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="35">
+        <f>IF(NOT(AND($B19&lt;&gt;"",ISNUMBER($D19))),"",IF($K19="No","Skip it",IF(N($E19)=0,"Find the usual price",IF($D19&gt;=$E19,"Not a deal",IF(N($O19)&gt;0.005,"Deal, but the plan costs more",IF($L19&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q19" s="1" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="56" t="n"/>
+      <c r="C20" s="59" t="n"/>
+      <c r="D20" s="60" t="n"/>
+      <c r="E20" s="60" t="n"/>
+      <c r="F20" s="65" t="n"/>
+      <c r="G20" s="60" t="n"/>
+      <c r="H20" s="59" t="n"/>
+      <c r="I20" s="63" t="n"/>
+      <c r="J20" s="60" t="n"/>
+      <c r="K20" s="59" t="n"/>
+      <c r="L20" s="22">
+        <f>IF(AND(AND($B20&lt;&gt;"",ISNUMBER($D20)),N($E20)&gt;0),($E20-$D20)/$E20,"")</f>
+        <v/>
+      </c>
+      <c r="M20" s="21">
+        <f>IF(AND($B20&lt;&gt;"",ISNUMBER($D20)),$D20*(1+N($F20))+N($G20),"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="21">
+        <f>IF(AND(AND($B20&lt;&gt;"",ISNUMBER($D20)),AND(N($I20)&gt;0,N($J20)&gt;0)),$I20*$J20,"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="21">
+        <f>IF(ISNUMBER($N20),MAX(0,$N20-$M20),"")</f>
+        <v/>
+      </c>
+      <c r="P20" s="33">
+        <f>IF(NOT(AND($B20&lt;&gt;"",ISNUMBER($D20))),"",IF($K20="No","Skip it",IF(N($E20)=0,"Find the usual price",IF($D20&gt;=$E20,"Not a deal",IF(N($O20)&gt;0.005,"Deal, but the plan costs more",IF($L20&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q20" s="1" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="57" t="n"/>
+      <c r="C21" s="61" t="n"/>
+      <c r="D21" s="62" t="n"/>
+      <c r="E21" s="62" t="n"/>
+      <c r="F21" s="70" t="n"/>
+      <c r="G21" s="62" t="n"/>
+      <c r="H21" s="61" t="n"/>
+      <c r="I21" s="68" t="n"/>
+      <c r="J21" s="62" t="n"/>
+      <c r="K21" s="61" t="n"/>
+      <c r="L21" s="25">
+        <f>IF(AND(AND($B21&lt;&gt;"",ISNUMBER($D21)),N($E21)&gt;0),($E21-$D21)/$E21,"")</f>
+        <v/>
+      </c>
+      <c r="M21" s="24">
+        <f>IF(AND($B21&lt;&gt;"",ISNUMBER($D21)),$D21*(1+N($F21))+N($G21),"")</f>
+        <v/>
+      </c>
+      <c r="N21" s="24">
+        <f>IF(AND(AND($B21&lt;&gt;"",ISNUMBER($D21)),AND(N($I21)&gt;0,N($J21)&gt;0)),$I21*$J21,"")</f>
+        <v/>
+      </c>
+      <c r="O21" s="24">
+        <f>IF(ISNUMBER($N21),MAX(0,$N21-$M21),"")</f>
+        <v/>
+      </c>
+      <c r="P21" s="35">
+        <f>IF(NOT(AND($B21&lt;&gt;"",ISNUMBER($D21))),"",IF($K21="No","Skip it",IF(N($E21)=0,"Find the usual price",IF($D21&gt;=$E21,"Not a deal",IF(N($O21)&gt;0.005,"Deal, but the plan costs more",IF($L21&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q21" s="1" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="56" t="n"/>
+      <c r="C22" s="59" t="n"/>
+      <c r="D22" s="60" t="n"/>
+      <c r="E22" s="60" t="n"/>
+      <c r="F22" s="65" t="n"/>
+      <c r="G22" s="60" t="n"/>
+      <c r="H22" s="59" t="n"/>
+      <c r="I22" s="63" t="n"/>
+      <c r="J22" s="60" t="n"/>
+      <c r="K22" s="59" t="n"/>
+      <c r="L22" s="22">
+        <f>IF(AND(AND($B22&lt;&gt;"",ISNUMBER($D22)),N($E22)&gt;0),($E22-$D22)/$E22,"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="21">
+        <f>IF(AND($B22&lt;&gt;"",ISNUMBER($D22)),$D22*(1+N($F22))+N($G22),"")</f>
+        <v/>
+      </c>
+      <c r="N22" s="21">
+        <f>IF(AND(AND($B22&lt;&gt;"",ISNUMBER($D22)),AND(N($I22)&gt;0,N($J22)&gt;0)),$I22*$J22,"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="21">
+        <f>IF(ISNUMBER($N22),MAX(0,$N22-$M22),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="33">
+        <f>IF(NOT(AND($B22&lt;&gt;"",ISNUMBER($D22))),"",IF($K22="No","Skip it",IF(N($E22)=0,"Find the usual price",IF($D22&gt;=$E22,"Not a deal",IF(N($O22)&gt;0.005,"Deal, but the plan costs more",IF($L22&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q22" s="1" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="57" t="n"/>
+      <c r="C23" s="61" t="n"/>
+      <c r="D23" s="62" t="n"/>
+      <c r="E23" s="62" t="n"/>
+      <c r="F23" s="70" t="n"/>
+      <c r="G23" s="62" t="n"/>
+      <c r="H23" s="61" t="n"/>
+      <c r="I23" s="68" t="n"/>
+      <c r="J23" s="62" t="n"/>
+      <c r="K23" s="61" t="n"/>
+      <c r="L23" s="25">
+        <f>IF(AND(AND($B23&lt;&gt;"",ISNUMBER($D23)),N($E23)&gt;0),($E23-$D23)/$E23,"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="24">
+        <f>IF(AND($B23&lt;&gt;"",ISNUMBER($D23)),$D23*(1+N($F23))+N($G23),"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="24">
+        <f>IF(AND(AND($B23&lt;&gt;"",ISNUMBER($D23)),AND(N($I23)&gt;0,N($J23)&gt;0)),$I23*$J23,"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="24">
+        <f>IF(ISNUMBER($N23),MAX(0,$N23-$M23),"")</f>
+        <v/>
+      </c>
+      <c r="P23" s="35">
+        <f>IF(NOT(AND($B23&lt;&gt;"",ISNUMBER($D23))),"",IF($K23="No","Skip it",IF(N($E23)=0,"Find the usual price",IF($D23&gt;=$E23,"Not a deal",IF(N($O23)&gt;0.005,"Deal, but the plan costs more",IF($L23&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q23" s="1" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="1" t="n"/>
+      <c r="B24" s="56" t="n"/>
+      <c r="C24" s="59" t="n"/>
+      <c r="D24" s="60" t="n"/>
+      <c r="E24" s="60" t="n"/>
+      <c r="F24" s="65" t="n"/>
+      <c r="G24" s="60" t="n"/>
+      <c r="H24" s="59" t="n"/>
+      <c r="I24" s="63" t="n"/>
+      <c r="J24" s="60" t="n"/>
+      <c r="K24" s="59" t="n"/>
+      <c r="L24" s="22">
+        <f>IF(AND(AND($B24&lt;&gt;"",ISNUMBER($D24)),N($E24)&gt;0),($E24-$D24)/$E24,"")</f>
+        <v/>
+      </c>
+      <c r="M24" s="21">
+        <f>IF(AND($B24&lt;&gt;"",ISNUMBER($D24)),$D24*(1+N($F24))+N($G24),"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="21">
+        <f>IF(AND(AND($B24&lt;&gt;"",ISNUMBER($D24)),AND(N($I24)&gt;0,N($J24)&gt;0)),$I24*$J24,"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="21">
+        <f>IF(ISNUMBER($N24),MAX(0,$N24-$M24),"")</f>
+        <v/>
+      </c>
+      <c r="P24" s="33">
+        <f>IF(NOT(AND($B24&lt;&gt;"",ISNUMBER($D24))),"",IF($K24="No","Skip it",IF(N($E24)=0,"Find the usual price",IF($D24&gt;=$E24,"Not a deal",IF(N($O24)&gt;0.005,"Deal, but the plan costs more",IF($L24&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q24" s="1" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="57" t="n"/>
+      <c r="C25" s="61" t="n"/>
+      <c r="D25" s="62" t="n"/>
+      <c r="E25" s="62" t="n"/>
+      <c r="F25" s="70" t="n"/>
+      <c r="G25" s="62" t="n"/>
+      <c r="H25" s="61" t="n"/>
+      <c r="I25" s="68" t="n"/>
+      <c r="J25" s="62" t="n"/>
+      <c r="K25" s="61" t="n"/>
+      <c r="L25" s="25">
+        <f>IF(AND(AND($B25&lt;&gt;"",ISNUMBER($D25)),N($E25)&gt;0),($E25-$D25)/$E25,"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="24">
+        <f>IF(AND($B25&lt;&gt;"",ISNUMBER($D25)),$D25*(1+N($F25))+N($G25),"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="24">
+        <f>IF(AND(AND($B25&lt;&gt;"",ISNUMBER($D25)),AND(N($I25)&gt;0,N($J25)&gt;0)),$I25*$J25,"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="24">
+        <f>IF(ISNUMBER($N25),MAX(0,$N25-$M25),"")</f>
+        <v/>
+      </c>
+      <c r="P25" s="35">
+        <f>IF(NOT(AND($B25&lt;&gt;"",ISNUMBER($D25))),"",IF($K25="No","Skip it",IF(N($E25)=0,"Find the usual price",IF($D25&gt;=$E25,"Not a deal",IF(N($O25)&gt;0.005,"Deal, but the plan costs more",IF($L25&lt;'Deal Check'!$M$4,"Small deal","Real deal"))))))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="1" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n"/>
+      <c r="B26" s="1" t="n"/>
+      <c r="C26" s="1" t="n"/>
+      <c r="D26" s="1" t="n"/>
+      <c r="E26" s="1" t="n"/>
+      <c r="F26" s="1" t="n"/>
+      <c r="G26" s="1" t="n"/>
+      <c r="H26" s="1" t="n"/>
+      <c r="I26" s="1" t="n"/>
+      <c r="J26" s="1" t="n"/>
+      <c r="K26" s="1" t="n"/>
+      <c r="L26" s="1" t="n"/>
+      <c r="M26" s="1" t="n"/>
+      <c r="N26" s="1" t="n"/>
+      <c r="O26" s="1" t="n"/>
+      <c r="P26" s="1" t="n"/>
+      <c r="Q26" s="1" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="n"/>
+      <c r="E27" s="1" t="n"/>
+      <c r="F27" s="1" t="n"/>
+      <c r="G27" s="1" t="n"/>
+      <c r="H27" s="1" t="n"/>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="1" t="n"/>
+      <c r="K27" s="1" t="n"/>
+      <c r="L27" s="1" t="n"/>
+      <c r="M27" s="1" t="n"/>
+      <c r="N27" s="1" t="n"/>
+      <c r="O27" s="1" t="n"/>
+      <c r="P27" s="1" t="n"/>
+      <c r="Q27" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="B5:P25"/>
+  <conditionalFormatting sqref="H6:H25">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+      <formula>"Cash / debit"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="6">
+      <formula>"Credit card"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Pay-in-4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>"Monthly BNPL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>"Store financing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"Gift card"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="7">
+      <formula>"Other"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6:K25">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="3">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="2">
+      <formula>"Maybe"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="7">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P6:P25">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="3">
+      <formula>"Real deal"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="2">
+      <formula>"Small deal"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="1">
+      <formula>"Deal, but the plan costs more"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="1">
+      <formula>"Not a deal"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="7">
+      <formula>"Skip it"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="6">
+      <formula>"Find the usual price"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O6:O25">
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>AND(ISNUMBER($O6),$O6&gt;0.005)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="H6:H25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Settings!$C$14:$C$21</formula1>
+    </dataValidation>
+    <dataValidation sqref="K6:K25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,Maybe,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="0026302A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -8529,7 +9738,7 @@
         <f>IFERROR(INDEX('Holiday Payments'!$M$6:$M$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,1),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
-      <c r="D22" s="73">
+      <c r="D22" s="74">
         <f>IFERROR(INDEX('Holiday Payments'!$Q$6:$Q$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,1),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
@@ -8550,7 +9759,7 @@
         <f>IFERROR(INDEX('Holiday Payments'!$M$6:$M$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,2),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
-      <c r="D23" s="73">
+      <c r="D23" s="74">
         <f>IFERROR(INDEX('Holiday Payments'!$Q$6:$Q$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,2),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
@@ -8571,7 +9780,7 @@
         <f>IFERROR(INDEX('Holiday Payments'!$M$6:$M$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,3),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
-      <c r="D24" s="73">
+      <c r="D24" s="74">
         <f>IFERROR(INDEX('Holiday Payments'!$Q$6:$Q$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,3),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
@@ -8592,7 +9801,7 @@
         <f>IFERROR(INDEX('Holiday Payments'!$M$6:$M$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,4),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
-      <c r="D25" s="73">
+      <c r="D25" s="74">
         <f>IFERROR(INDEX('Holiday Payments'!$Q$6:$Q$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,4),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
@@ -8613,7 +9822,7 @@
         <f>IFERROR(INDEX('Holiday Payments'!$M$6:$M$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,5),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
-      <c r="D26" s="73">
+      <c r="D26" s="74">
         <f>IFERROR(INDEX('Holiday Payments'!$Q$6:$Q$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,5),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
@@ -8634,7 +9843,7 @@
         <f>IFERROR(INDEX('Holiday Payments'!$M$6:$M$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,6),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>
-      <c r="D27" s="73">
+      <c r="D27" s="74">
         <f>IFERROR(INDEX('Holiday Payments'!$Q$6:$Q$25,MATCH(LARGE('Holiday Payments'!$W$6:$W$25,6),'Holiday Payments'!$W$6:$W$25,0)),"")</f>
         <v/>
       </c>

</xml_diff>